<commit_message>
Add 6/30 data; update total to 50組 (42跨型態); add 文案效果小結 slide
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/志明AI實驗數據_6_1-6_30.xlsx
+++ b/志明AI實驗數據_6_1-6_30.xlsx
@@ -124,10 +124,10 @@
         <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
-        <a:font script="Hang" typeface="맑은 고딕"/>
-        <a:font script="Hans" typeface="宋体"/>
-        <a:font script="Hant" typeface="新細明體"/>
+        <a:font script="Jpan" typeface="ï¼­ï¼³ ï¼°ã´ã·ãã¯"/>
+        <a:font script="Hang" typeface="ë§ì ê³ ë"/>
+        <a:font script="Hans" typeface="å®ä½"/>
+        <a:font script="Hant" typeface="æ°ç´°æé«"/>
         <a:font script="Arab" typeface="Times New Roman"/>
         <a:font script="Hebr" typeface="Times New Roman"/>
         <a:font script="Thai" typeface="Tahoma"/>
@@ -159,10 +159,10 @@
         <a:latin typeface="Calibri"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
-        <a:font script="Hang" typeface="맑은 고딕"/>
-        <a:font script="Hans" typeface="宋体"/>
-        <a:font script="Hant" typeface="新細明體"/>
+        <a:font script="Jpan" typeface="ï¼­ï¼³ ï¼°ã´ã·ãã¯"/>
+        <a:font script="Hang" typeface="ë§ì ê³ ë"/>
+        <a:font script="Hans" typeface="å®ä½"/>
+        <a:font script="Hant" typeface="æ°ç´°æé«"/>
         <a:font script="Arab" typeface="Arial"/>
         <a:font script="Hebr" typeface="Arial"/>
         <a:font script="Thai" typeface="Tahoma"/>
@@ -400,7 +400,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:N39"/>
+  <dimension ref="A1:N43"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -2118,9 +2118,173 @@
         <v>3變體取最佳圖像(C)vs連結(B)</v>
       </c>
     </row>
+    <row r="40">
+      <c r="A40">
+        <v>39</v>
+      </c>
+      <c r="B40" t="str">
+        <v>6/30</v>
+      </c>
+      <c r="C40" t="str">
+        <v>梅雨季最濕（since 2012）</v>
+      </c>
+      <c r="D40">
+        <v>562</v>
+      </c>
+      <c r="E40">
+        <v>187</v>
+      </c>
+      <c r="F40">
+        <v>3.01</v>
+      </c>
+      <c r="G40">
+        <v>6</v>
+      </c>
+      <c r="H40">
+        <v>0</v>
+      </c>
+      <c r="J40" t="str">
+        <v>環境</v>
+      </c>
+      <c r="K40">
+        <v>1.068</v>
+      </c>
+      <c r="L40">
+        <v>0</v>
+      </c>
+      <c r="M40">
+        <v>1.068</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41">
+        <v>40</v>
+      </c>
+      <c r="B41" t="str">
+        <v>6/30</v>
+      </c>
+      <c r="C41" t="str">
+        <v>三鶯線通車</v>
+      </c>
+      <c r="D41">
+        <v>367</v>
+      </c>
+      <c r="E41">
+        <v>232</v>
+      </c>
+      <c r="F41">
+        <v>1.58</v>
+      </c>
+      <c r="G41">
+        <v>2</v>
+      </c>
+      <c r="H41">
+        <v>4</v>
+      </c>
+      <c r="I41">
+        <v>4</v>
+      </c>
+      <c r="J41" t="str">
+        <v>社會</v>
+      </c>
+      <c r="K41">
+        <v>0.545</v>
+      </c>
+      <c r="L41">
+        <v>1.724</v>
+      </c>
+      <c r="M41">
+        <v>-1.179</v>
+      </c>
+      <c r="N41" t="str">
+        <v>連結互動勝（心情4 vs 2）</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42">
+        <v>41</v>
+      </c>
+      <c r="B42" t="str">
+        <v>6/30</v>
+      </c>
+      <c r="C42" t="str">
+        <v>阿里山鐵道闖入</v>
+      </c>
+      <c r="D42">
+        <v>2027</v>
+      </c>
+      <c r="E42">
+        <v>564</v>
+      </c>
+      <c r="F42">
+        <v>3.59</v>
+      </c>
+      <c r="G42">
+        <v>15</v>
+      </c>
+      <c r="H42">
+        <v>2</v>
+      </c>
+      <c r="I42">
+        <v>26</v>
+      </c>
+      <c r="J42" t="str">
+        <v>公安</v>
+      </c>
+      <c r="K42">
+        <v>0.74</v>
+      </c>
+      <c r="L42">
+        <v>0.355</v>
+      </c>
+      <c r="M42">
+        <v>0.385</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43">
+        <v>42</v>
+      </c>
+      <c r="B43" t="str">
+        <v>6/30</v>
+      </c>
+      <c r="C43" t="str">
+        <v>加密貨幣監管法</v>
+      </c>
+      <c r="D43">
+        <v>259</v>
+      </c>
+      <c r="E43">
+        <v>168</v>
+      </c>
+      <c r="F43">
+        <v>1.54</v>
+      </c>
+      <c r="G43">
+        <v>0</v>
+      </c>
+      <c r="H43">
+        <v>0</v>
+      </c>
+      <c r="I43">
+        <v>1</v>
+      </c>
+      <c r="J43" t="str">
+        <v>財經</v>
+      </c>
+      <c r="K43">
+        <v>0</v>
+      </c>
+      <c r="L43">
+        <v>0</v>
+      </c>
+      <c r="M43">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:N39"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:N43"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>